<commit_message>
Preliminary hfs treatment; fixes to codes; new level 658
</commit_message>
<xml_diff>
--- a/LineClass/levels_pub.xlsx
+++ b/LineClass/levels_pub.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\UMD\AI\as-ai\LineClass\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF016F6-7F02-423B-B40B-A694DD697E14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4F47FBE-A511-4912-A02C-3CC743A5B83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1425" yWindow="1425" windowWidth="47115" windowHeight="17505" xr2:uid="{68E62A3F-E4FB-447B-97FA-80FE60CCF832}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="43920" windowHeight="17505" xr2:uid="{68E62A3F-E4FB-447B-97FA-80FE60CCF832}"/>
   </bookViews>
   <sheets>
     <sheet name="levels_pub" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7296" uniqueCount="896">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7303" uniqueCount="903">
   <si>
     <t>conf</t>
   </si>
@@ -2724,6 +2724,27 @@
   </si>
   <si>
     <t>059003.000624</t>
+  </si>
+  <si>
+    <t>059003.000642</t>
+  </si>
+  <si>
+    <t>059003.000676</t>
+  </si>
+  <si>
+    <t>059003.000652</t>
+  </si>
+  <si>
+    <t>059003.000680</t>
+  </si>
+  <si>
+    <t>059003.000678</t>
+  </si>
+  <si>
+    <t>059003.000673</t>
+  </si>
+  <si>
+    <t>059003.000625</t>
   </si>
 </sst>
 </file>
@@ -3592,7 +3613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29751ECF-5867-4DFC-949B-BE61CEB11EBC}">
-  <sheetPr codeName="Sheet1"/>
+  <sheetPr codeName="Sheet1" filterMode="1"/>
   <dimension ref="A1:S1037"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3676,7 +3697,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3717,7 +3738,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3749,7 +3770,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -3781,7 +3802,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>16</v>
       </c>
@@ -3813,7 +3834,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3854,7 +3875,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -3904,7 +3925,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -3945,7 +3966,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>16</v>
       </c>
@@ -3995,7 +4016,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -4036,7 +4057,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -4086,7 +4107,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -4136,7 +4157,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -4186,7 +4207,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>16</v>
       </c>
@@ -4218,7 +4239,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -4268,7 +4289,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -4327,7 +4348,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -4359,7 +4380,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -4409,7 +4430,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -4459,7 +4480,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -4509,7 +4530,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -4550,7 +4571,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -4591,7 +4612,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -4632,7 +4653,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -4682,7 +4703,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>16</v>
       </c>
@@ -4732,7 +4753,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>16</v>
       </c>
@@ -4782,7 +4803,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>16</v>
       </c>
@@ -4832,7 +4853,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>16</v>
       </c>
@@ -4873,7 +4894,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -4914,7 +4935,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>16</v>
       </c>
@@ -4955,7 +4976,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>16</v>
       </c>
@@ -4987,7 +5008,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>16</v>
       </c>
@@ -5019,7 +5040,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>16</v>
       </c>
@@ -5069,7 +5090,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>16</v>
       </c>
@@ -5110,7 +5131,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>16</v>
       </c>
@@ -5160,7 +5181,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>16</v>
       </c>
@@ -5210,7 +5231,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>16</v>
       </c>
@@ -5260,7 +5281,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>16</v>
       </c>
@@ -5310,7 +5331,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>16</v>
       </c>
@@ -5360,7 +5381,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>16</v>
       </c>
@@ -5410,7 +5431,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -5460,7 +5481,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>16</v>
       </c>
@@ -5502,7 +5523,7 @@
       </c>
       <c r="S42"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>16</v>
       </c>
@@ -5552,7 +5573,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>16</v>
       </c>
@@ -5602,7 +5623,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>16</v>
       </c>
@@ -5652,7 +5673,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>16</v>
       </c>
@@ -5702,7 +5723,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>16</v>
       </c>
@@ -5752,7 +5773,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>16</v>
       </c>
@@ -5802,7 +5823,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>16</v>
       </c>
@@ -5852,7 +5873,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>16</v>
       </c>
@@ -5902,7 +5923,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>16</v>
       </c>
@@ -5952,7 +5973,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>16</v>
       </c>
@@ -6002,7 +6023,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>16</v>
       </c>
@@ -6052,7 +6073,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>16</v>
       </c>
@@ -6093,7 +6114,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>16</v>
       </c>
@@ -6143,7 +6164,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>16</v>
       </c>
@@ -6193,7 +6214,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>16</v>
       </c>
@@ -6235,7 +6256,7 @@
       </c>
       <c r="S57"/>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>16</v>
       </c>
@@ -6294,7 +6315,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>16</v>
       </c>
@@ -6344,7 +6365,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>16</v>
       </c>
@@ -6394,7 +6415,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>16</v>
       </c>
@@ -6444,7 +6465,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>16</v>
       </c>
@@ -6503,7 +6524,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>16</v>
       </c>
@@ -6553,7 +6574,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>16</v>
       </c>
@@ -6603,7 +6624,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>16</v>
       </c>
@@ -6662,7 +6683,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>16</v>
       </c>
@@ -6712,7 +6733,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>16</v>
       </c>
@@ -6762,7 +6783,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>16</v>
       </c>
@@ -6812,7 +6833,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>16</v>
       </c>
@@ -6862,7 +6883,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>16</v>
       </c>
@@ -6912,7 +6933,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>16</v>
       </c>
@@ -6962,7 +6983,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>16</v>
       </c>
@@ -7012,7 +7033,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>16</v>
       </c>
@@ -7054,7 +7075,7 @@
       </c>
       <c r="S73"/>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>16</v>
       </c>
@@ -7104,7 +7125,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>16</v>
       </c>
@@ -7154,7 +7175,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -7204,7 +7225,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>16</v>
       </c>
@@ -7254,7 +7275,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>16</v>
       </c>
@@ -7304,7 +7325,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>16</v>
       </c>
@@ -7354,7 +7375,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>16</v>
       </c>
@@ -7404,7 +7425,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="81" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>16</v>
       </c>
@@ -7445,7 +7466,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="82" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>16</v>
       </c>
@@ -7504,7 +7525,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="83" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -7554,7 +7575,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="84" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>16</v>
       </c>
@@ -7604,7 +7625,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="85" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>16</v>
       </c>
@@ -7654,7 +7675,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="86" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -7704,7 +7725,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="87" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>16</v>
       </c>
@@ -7754,7 +7775,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="88" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>16</v>
       </c>
@@ -7804,7 +7825,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="89" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>16</v>
       </c>
@@ -7854,7 +7875,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="90" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>16</v>
       </c>
@@ -7904,7 +7925,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="91" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>16</v>
       </c>
@@ -7954,7 +7975,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="92" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>16</v>
       </c>
@@ -7995,7 +8016,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="93" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>16</v>
       </c>
@@ -8045,7 +8066,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="94" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>16</v>
       </c>
@@ -8095,7 +8116,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="95" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>16</v>
       </c>
@@ -8145,7 +8166,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="96" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>16</v>
       </c>
@@ -8195,7 +8216,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>16</v>
       </c>
@@ -8236,7 +8257,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>16</v>
       </c>
@@ -8286,7 +8307,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>16</v>
       </c>
@@ -8336,7 +8357,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>16</v>
       </c>
@@ -8386,7 +8407,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>16</v>
       </c>
@@ -8436,7 +8457,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>16</v>
       </c>
@@ -8495,7 +8516,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>16</v>
       </c>
@@ -8537,7 +8558,7 @@
       </c>
       <c r="S103"/>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>16</v>
       </c>
@@ -8587,7 +8608,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>16</v>
       </c>
@@ -8637,7 +8658,7 @@
         <v>556</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>16</v>
       </c>
@@ -8687,7 +8708,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>16</v>
       </c>
@@ -8737,7 +8758,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>16</v>
       </c>
@@ -8787,7 +8808,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -8837,7 +8858,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>16</v>
       </c>
@@ -8887,7 +8908,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>16</v>
       </c>
@@ -8938,7 +8959,7 @@
       </c>
       <c r="S111"/>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>16</v>
       </c>
@@ -8970,7 +8991,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>16</v>
       </c>
@@ -9020,7 +9041,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="114" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -9070,7 +9091,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>16</v>
       </c>
@@ -9112,7 +9133,7 @@
       </c>
       <c r="S115"/>
     </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>16</v>
       </c>
@@ -9162,7 +9183,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>16</v>
       </c>
@@ -9204,7 +9225,7 @@
       </c>
       <c r="S117"/>
     </row>
-    <row r="118" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>16</v>
       </c>
@@ -9246,7 +9267,7 @@
       </c>
       <c r="S118"/>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>16</v>
       </c>
@@ -9296,7 +9317,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>16</v>
       </c>
@@ -9346,7 +9367,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>16</v>
       </c>
@@ -9396,7 +9417,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="122" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>16</v>
       </c>
@@ -9446,7 +9467,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>16</v>
       </c>
@@ -9496,7 +9517,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>16</v>
       </c>
@@ -9546,7 +9567,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>16</v>
       </c>
@@ -9596,7 +9617,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -9646,7 +9667,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>16</v>
       </c>
@@ -9688,7 +9709,7 @@
       </c>
       <c r="S127"/>
     </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>16</v>
       </c>
@@ -9738,7 +9759,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>16</v>
       </c>
@@ -9780,7 +9801,7 @@
       </c>
       <c r="S129"/>
     </row>
-    <row r="130" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>16</v>
       </c>
@@ -9830,7 +9851,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>16</v>
       </c>
@@ -9872,7 +9893,7 @@
       </c>
       <c r="S131"/>
     </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>16</v>
       </c>
@@ -9922,7 +9943,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>16</v>
       </c>
@@ -9972,7 +9993,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="134" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>16</v>
       </c>
@@ -10031,7 +10052,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>16</v>
       </c>
@@ -10081,7 +10102,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>16</v>
       </c>
@@ -10131,7 +10152,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>16</v>
       </c>
@@ -10190,7 +10211,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="138" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>16</v>
       </c>
@@ -10232,7 +10253,7 @@
       </c>
       <c r="S138"/>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>16</v>
       </c>
@@ -10274,7 +10295,7 @@
       </c>
       <c r="S139"/>
     </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>16</v>
       </c>
@@ -10324,7 +10345,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>16</v>
       </c>
@@ -10374,7 +10395,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="142" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>16</v>
       </c>
@@ -10425,7 +10446,7 @@
       </c>
       <c r="S142"/>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>16</v>
       </c>
@@ -10475,7 +10496,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>16</v>
       </c>
@@ -10525,7 +10546,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="145" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>16</v>
       </c>
@@ -10575,7 +10596,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="146" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>16</v>
       </c>
@@ -10625,7 +10646,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="147" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>16</v>
       </c>
@@ -10675,7 +10696,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="148" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>16</v>
       </c>
@@ -10725,7 +10746,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="149" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>16</v>
       </c>
@@ -10775,7 +10796,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="150" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>16</v>
       </c>
@@ -10825,7 +10846,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="151" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>16</v>
       </c>
@@ -10884,7 +10905,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="152" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>16</v>
       </c>
@@ -10934,7 +10955,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="153" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>16</v>
       </c>
@@ -10984,7 +11005,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="154" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>16</v>
       </c>
@@ -11034,7 +11055,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="155" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>16</v>
       </c>
@@ -11084,7 +11105,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="156" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>16</v>
       </c>
@@ -11134,7 +11155,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="157" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>16</v>
       </c>
@@ -11184,7 +11205,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="158" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>16</v>
       </c>
@@ -11234,7 +11255,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="159" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>16</v>
       </c>
@@ -11275,7 +11296,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="160" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>16</v>
       </c>
@@ -11325,7 +11346,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="161" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>16</v>
       </c>
@@ -11375,7 +11396,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="162" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>16</v>
       </c>
@@ -11425,7 +11446,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>16</v>
       </c>
@@ -11475,7 +11496,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>16</v>
       </c>
@@ -11525,7 +11546,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="165" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>16</v>
       </c>
@@ -11575,7 +11596,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="166" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>16</v>
       </c>
@@ -11625,7 +11646,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="167" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>16</v>
       </c>
@@ -11675,7 +11696,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="168" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>16</v>
       </c>
@@ -11725,7 +11746,7 @@
         <v>692</v>
       </c>
     </row>
-    <row r="169" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>16</v>
       </c>
@@ -11767,7 +11788,7 @@
       </c>
       <c r="S169"/>
     </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>16</v>
       </c>
@@ -11817,7 +11838,7 @@
         <v>718</v>
       </c>
     </row>
-    <row r="171" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>16</v>
       </c>
@@ -11867,7 +11888,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="172" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>16</v>
       </c>
@@ -11917,7 +11938,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="173" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>16</v>
       </c>
@@ -11959,7 +11980,7 @@
       </c>
       <c r="S173"/>
     </row>
-    <row r="174" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>16</v>
       </c>
@@ -12009,7 +12030,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="175" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>16</v>
       </c>
@@ -12051,7 +12072,7 @@
       </c>
       <c r="S175"/>
     </row>
-    <row r="176" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>16</v>
       </c>
@@ -12101,7 +12122,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="177" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>16</v>
       </c>
@@ -12151,7 +12172,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>16</v>
       </c>
@@ -12201,7 +12222,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="179" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>16</v>
       </c>
@@ -12251,7 +12272,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="180" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>16</v>
       </c>
@@ -12293,7 +12314,7 @@
       </c>
       <c r="S180"/>
     </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>16</v>
       </c>
@@ -12352,7 +12373,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="182" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>16</v>
       </c>
@@ -12402,7 +12423,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="183" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>16</v>
       </c>
@@ -12452,7 +12473,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="184" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>16</v>
       </c>
@@ -12494,7 +12515,7 @@
       </c>
       <c r="S184"/>
     </row>
-    <row r="185" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>16</v>
       </c>
@@ -12544,7 +12565,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="186" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>16</v>
       </c>
@@ -12594,7 +12615,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="187" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>16</v>
       </c>
@@ -12636,7 +12657,7 @@
       </c>
       <c r="S187"/>
     </row>
-    <row r="188" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>16</v>
       </c>
@@ -12677,7 +12698,7 @@
         <v>1.1559999999999999</v>
       </c>
     </row>
-    <row r="189" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>16</v>
       </c>
@@ -12718,7 +12739,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="190" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>16</v>
       </c>
@@ -12768,7 +12789,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="191" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>16</v>
       </c>
@@ -12818,7 +12839,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="192" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>16</v>
       </c>
@@ -12867,8 +12888,11 @@
       <c r="R192">
         <v>0.88200000000000001</v>
       </c>
-    </row>
-    <row r="193" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="S192" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="193" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>16</v>
       </c>
@@ -12918,7 +12942,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="194" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>16</v>
       </c>
@@ -12968,7 +12992,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="195" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>16</v>
       </c>
@@ -13018,7 +13042,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="196" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>16</v>
       </c>
@@ -13060,7 +13084,7 @@
       </c>
       <c r="S196"/>
     </row>
-    <row r="197" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>16</v>
       </c>
@@ -13110,7 +13134,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="198" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>16</v>
       </c>
@@ -13151,7 +13175,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="199" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>16</v>
       </c>
@@ -13201,7 +13225,7 @@
         <v>774</v>
       </c>
     </row>
-    <row r="200" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>16</v>
       </c>
@@ -13243,7 +13267,7 @@
       </c>
       <c r="S200"/>
     </row>
-    <row r="201" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>16</v>
       </c>
@@ -13293,7 +13317,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="202" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>16</v>
       </c>
@@ -13335,7 +13359,7 @@
       </c>
       <c r="S202"/>
     </row>
-    <row r="203" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>16</v>
       </c>
@@ -13377,7 +13401,7 @@
       </c>
       <c r="S203"/>
     </row>
-    <row r="204" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>16</v>
       </c>
@@ -13409,7 +13433,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="205" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>16</v>
       </c>
@@ -13460,7 +13484,7 @@
       </c>
       <c r="S205"/>
     </row>
-    <row r="206" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>16</v>
       </c>
@@ -13510,7 +13534,7 @@
         <v>1.1870000000000001</v>
       </c>
     </row>
-    <row r="207" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>16</v>
       </c>
@@ -13542,7 +13566,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="208" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>16</v>
       </c>
@@ -13592,7 +13616,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="209" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>16</v>
       </c>
@@ -13634,7 +13658,7 @@
       </c>
       <c r="S209"/>
     </row>
-    <row r="210" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>16</v>
       </c>
@@ -13676,7 +13700,7 @@
       </c>
       <c r="S210"/>
     </row>
-    <row r="211" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>16</v>
       </c>
@@ -13717,7 +13741,7 @@
         <v>1.282</v>
       </c>
     </row>
-    <row r="212" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>16</v>
       </c>
@@ -13767,7 +13791,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="213" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>16</v>
       </c>
@@ -13817,7 +13841,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="214" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>16</v>
       </c>
@@ -13859,7 +13883,7 @@
       </c>
       <c r="S214"/>
     </row>
-    <row r="215" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>16</v>
       </c>
@@ -13909,7 +13933,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="216" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>16</v>
       </c>
@@ -13951,7 +13975,7 @@
       </c>
       <c r="S216"/>
     </row>
-    <row r="217" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>16</v>
       </c>
@@ -14001,7 +14025,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="218" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>16</v>
       </c>
@@ -14043,7 +14067,7 @@
       </c>
       <c r="S218"/>
     </row>
-    <row r="219" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>16</v>
       </c>
@@ -14085,7 +14109,7 @@
       </c>
       <c r="S219"/>
     </row>
-    <row r="220" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>16</v>
       </c>
@@ -14135,7 +14159,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="221" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>16</v>
       </c>
@@ -14177,7 +14201,7 @@
       </c>
       <c r="S221"/>
     </row>
-    <row r="222" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>16</v>
       </c>
@@ -14227,7 +14251,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="223" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>16</v>
       </c>
@@ -14269,7 +14293,7 @@
       </c>
       <c r="S223"/>
     </row>
-    <row r="224" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>16</v>
       </c>
@@ -14311,7 +14335,7 @@
       </c>
       <c r="S224"/>
     </row>
-    <row r="225" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>16</v>
       </c>
@@ -14353,7 +14377,7 @@
       </c>
       <c r="S225"/>
     </row>
-    <row r="226" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>16</v>
       </c>
@@ -14403,7 +14427,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="227" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>16</v>
       </c>
@@ -14453,7 +14477,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="228" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>16</v>
       </c>
@@ -14495,7 +14519,7 @@
       </c>
       <c r="S228"/>
     </row>
-    <row r="229" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>16</v>
       </c>
@@ -14537,7 +14561,7 @@
       </c>
       <c r="S229"/>
     </row>
-    <row r="230" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>16</v>
       </c>
@@ -14579,7 +14603,7 @@
       </c>
       <c r="S230"/>
     </row>
-    <row r="231" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>16</v>
       </c>
@@ -14620,7 +14644,7 @@
         <v>1.143</v>
       </c>
     </row>
-    <row r="232" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>16</v>
       </c>
@@ -14653,7 +14677,7 @@
       </c>
       <c r="S232"/>
     </row>
-    <row r="233" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>16</v>
       </c>
@@ -14703,7 +14727,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="234" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>16</v>
       </c>
@@ -14753,7 +14777,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="235" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>16</v>
       </c>
@@ -14794,7 +14818,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="236" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>16</v>
       </c>
@@ -14844,7 +14868,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="237" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>16</v>
       </c>
@@ -14894,7 +14918,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="238" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>16</v>
       </c>
@@ -14944,7 +14968,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="239" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>16</v>
       </c>
@@ -14994,7 +15018,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="240" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>16</v>
       </c>
@@ -15044,7 +15068,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="241" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>16</v>
       </c>
@@ -15094,7 +15118,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="242" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>16</v>
       </c>
@@ -15144,7 +15168,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="243" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>16</v>
       </c>
@@ -15194,7 +15218,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="244" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>16</v>
       </c>
@@ -15244,7 +15268,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="245" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>16</v>
       </c>
@@ -15294,7 +15318,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="246" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>16</v>
       </c>
@@ -15344,7 +15368,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="247" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>16</v>
       </c>
@@ -15394,7 +15418,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="248" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>16</v>
       </c>
@@ -15444,7 +15468,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="249" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>16</v>
       </c>
@@ -15477,7 +15501,7 @@
       </c>
       <c r="S249"/>
     </row>
-    <row r="250" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>16</v>
       </c>
@@ -15527,7 +15551,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="251" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>16</v>
       </c>
@@ -15577,7 +15601,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="252" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>16</v>
       </c>
@@ -15627,7 +15651,7 @@
         <v>514</v>
       </c>
     </row>
-    <row r="253" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>16</v>
       </c>
@@ -15677,7 +15701,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="254" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>16</v>
       </c>
@@ -15727,7 +15751,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="255" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>16</v>
       </c>
@@ -15768,7 +15792,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="256" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>16</v>
       </c>
@@ -15818,7 +15842,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="257" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>16</v>
       </c>
@@ -15868,7 +15892,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="258" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>16</v>
       </c>
@@ -15918,7 +15942,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="259" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>16</v>
       </c>
@@ -15968,7 +15992,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="260" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>16</v>
       </c>
@@ -16018,7 +16042,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="261" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>16</v>
       </c>
@@ -16068,7 +16092,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="262" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>16</v>
       </c>
@@ -16118,7 +16142,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="263" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>16</v>
       </c>
@@ -16168,7 +16192,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="264" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>16</v>
       </c>
@@ -16218,7 +16242,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="265" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>16</v>
       </c>
@@ -16277,7 +16301,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="266" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>16</v>
       </c>
@@ -16327,7 +16351,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="267" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>16</v>
       </c>
@@ -16377,7 +16401,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="268" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>16</v>
       </c>
@@ -16427,7 +16451,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="269" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>16</v>
       </c>
@@ -16486,7 +16510,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="270" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>16</v>
       </c>
@@ -16527,7 +16551,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="271" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>16</v>
       </c>
@@ -16577,7 +16601,7 @@
         <v>569</v>
       </c>
     </row>
-    <row r="272" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>16</v>
       </c>
@@ -16618,7 +16642,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="273" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>16</v>
       </c>
@@ -16650,7 +16674,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="274" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>16</v>
       </c>
@@ -16700,7 +16724,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="275" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>16</v>
       </c>
@@ -16750,7 +16774,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="276" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>16</v>
       </c>
@@ -16800,7 +16824,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="277" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>16</v>
       </c>
@@ -16859,7 +16883,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="278" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>16</v>
       </c>
@@ -16909,7 +16933,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="279" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>16</v>
       </c>
@@ -16959,7 +16983,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="280" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>16</v>
       </c>
@@ -17009,7 +17033,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="281" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
         <v>16</v>
       </c>
@@ -17059,7 +17083,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="282" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
         <v>16</v>
       </c>
@@ -17109,7 +17133,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="283" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>16</v>
       </c>
@@ -17159,7 +17183,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="284" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
         <v>16</v>
       </c>
@@ -17209,7 +17233,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="285" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
         <v>16</v>
       </c>
@@ -17259,7 +17283,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="286" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>16</v>
       </c>
@@ -17309,7 +17333,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="287" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>16</v>
       </c>
@@ -17359,7 +17383,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="288" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
         <v>16</v>
       </c>
@@ -17409,7 +17433,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="289" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
         <v>16</v>
       </c>
@@ -17459,7 +17483,7 @@
         <v>645</v>
       </c>
     </row>
-    <row r="290" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
         <v>16</v>
       </c>
@@ -17492,7 +17516,7 @@
       </c>
       <c r="S290"/>
     </row>
-    <row r="291" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
         <v>16</v>
       </c>
@@ -17542,7 +17566,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="292" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
         <v>16</v>
       </c>
@@ -17592,7 +17616,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="293" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
         <v>16</v>
       </c>
@@ -17642,7 +17666,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="294" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
         <v>16</v>
       </c>
@@ -17692,7 +17716,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="295" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
         <v>16</v>
       </c>
@@ -17736,7 +17760,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="296" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
         <v>16</v>
       </c>
@@ -17778,7 +17802,7 @@
       </c>
       <c r="S296"/>
     </row>
-    <row r="297" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
         <v>16</v>
       </c>
@@ -17820,7 +17844,7 @@
       </c>
       <c r="S297"/>
     </row>
-    <row r="298" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
         <v>16</v>
       </c>
@@ -17870,7 +17894,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="299" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
         <v>16</v>
       </c>
@@ -17920,7 +17944,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="300" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
         <v>16</v>
       </c>
@@ -17970,7 +17994,7 @@
         <v>666</v>
       </c>
     </row>
-    <row r="301" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
         <v>16</v>
       </c>
@@ -18012,7 +18036,7 @@
       </c>
       <c r="S301"/>
     </row>
-    <row r="302" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
         <v>16</v>
       </c>
@@ -18062,7 +18086,7 @@
         <v>674</v>
       </c>
     </row>
-    <row r="303" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
         <v>16</v>
       </c>
@@ -18112,7 +18136,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="304" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>16</v>
       </c>
@@ -18162,7 +18186,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="305" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
         <v>16</v>
       </c>
@@ -18212,7 +18236,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="306" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>16</v>
       </c>
@@ -18253,7 +18277,7 @@
         <v>705</v>
       </c>
     </row>
-    <row r="307" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
         <v>16</v>
       </c>
@@ -18303,7 +18327,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="308" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>16</v>
       </c>
@@ -18344,7 +18368,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="309" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
         <v>16</v>
       </c>
@@ -18394,7 +18418,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="310" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
         <v>16</v>
       </c>
@@ -18444,7 +18468,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="311" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
         <v>16</v>
       </c>
@@ -18494,7 +18518,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="312" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
         <v>16</v>
       </c>
@@ -18544,7 +18568,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="313" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
         <v>16</v>
       </c>
@@ -18594,7 +18618,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="314" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
         <v>16</v>
       </c>
@@ -18644,7 +18668,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="315" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
         <v>16</v>
       </c>
@@ -18686,7 +18710,7 @@
       </c>
       <c r="S315"/>
     </row>
-    <row r="316" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
         <v>16</v>
       </c>
@@ -18719,7 +18743,7 @@
       </c>
       <c r="S316"/>
     </row>
-    <row r="317" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
         <v>16</v>
       </c>
@@ -18751,7 +18775,7 @@
         <v>0.98799999999999999</v>
       </c>
     </row>
-    <row r="318" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
         <v>16</v>
       </c>
@@ -18793,7 +18817,7 @@
       </c>
       <c r="S318"/>
     </row>
-    <row r="319" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
         <v>16</v>
       </c>
@@ -18843,7 +18867,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="320" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
         <v>16</v>
       </c>
@@ -18867,7 +18891,7 @@
       </c>
       <c r="S320"/>
     </row>
-    <row r="321" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
         <v>16</v>
       </c>
@@ -18900,7 +18924,7 @@
       </c>
       <c r="S321"/>
     </row>
-    <row r="322" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
         <v>16</v>
       </c>
@@ -18959,7 +18983,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="323" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
         <v>16</v>
       </c>
@@ -19009,7 +19033,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="324" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
         <v>16</v>
       </c>
@@ -19059,7 +19083,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="325" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
         <v>16</v>
       </c>
@@ -19100,7 +19124,7 @@
         <v>1.03</v>
       </c>
     </row>
-    <row r="326" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
         <v>16</v>
       </c>
@@ -19150,7 +19174,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="327" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
         <v>16</v>
       </c>
@@ -19200,7 +19224,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="328" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
         <v>16</v>
       </c>
@@ -19250,7 +19274,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="329" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
         <v>16</v>
       </c>
@@ -19300,7 +19324,7 @@
         <v>758</v>
       </c>
     </row>
-    <row r="330" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
         <v>16</v>
       </c>
@@ -19350,7 +19374,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="331" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
         <v>16</v>
       </c>
@@ -19409,7 +19433,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="332" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
         <v>16</v>
       </c>
@@ -19450,7 +19474,7 @@
         <v>1.252</v>
       </c>
     </row>
-    <row r="333" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
         <v>16</v>
       </c>
@@ -19492,7 +19516,7 @@
       </c>
       <c r="S333"/>
     </row>
-    <row r="334" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
         <v>16</v>
       </c>
@@ -19542,7 +19566,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="335" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
         <v>16</v>
       </c>
@@ -19592,7 +19616,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="336" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
         <v>16</v>
       </c>
@@ -19642,7 +19666,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="337" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
         <v>16</v>
       </c>
@@ -19692,7 +19716,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="338" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
         <v>16</v>
       </c>
@@ -19751,7 +19775,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="339" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
         <v>16</v>
       </c>
@@ -19801,7 +19825,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="340" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
         <v>16</v>
       </c>
@@ -19851,7 +19875,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="341" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
         <v>16</v>
       </c>
@@ -19884,7 +19908,7 @@
       </c>
       <c r="S341"/>
     </row>
-    <row r="342" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
         <v>16</v>
       </c>
@@ -19908,7 +19932,7 @@
       </c>
       <c r="S342"/>
     </row>
-    <row r="343" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
         <v>16</v>
       </c>
@@ -19941,7 +19965,7 @@
       </c>
       <c r="S343"/>
     </row>
-    <row r="344" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
         <v>16</v>
       </c>
@@ -19964,7 +19988,7 @@
         <v>1.147</v>
       </c>
     </row>
-    <row r="345" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
         <v>16</v>
       </c>
@@ -19997,7 +20021,7 @@
       </c>
       <c r="S345"/>
     </row>
-    <row r="346" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
         <v>16</v>
       </c>
@@ -20029,7 +20053,7 @@
         <v>1.1319999999999999</v>
       </c>
     </row>
-    <row r="347" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
         <v>16</v>
       </c>
@@ -20071,7 +20095,7 @@
       </c>
       <c r="S347"/>
     </row>
-    <row r="348" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
         <v>16</v>
       </c>
@@ -20104,7 +20128,7 @@
       </c>
       <c r="S348"/>
     </row>
-    <row r="349" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
         <v>16</v>
       </c>
@@ -20154,7 +20178,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="350" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
         <v>16</v>
       </c>
@@ -20196,7 +20220,7 @@
       </c>
       <c r="S350"/>
     </row>
-    <row r="351" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
         <v>16</v>
       </c>
@@ -20246,7 +20270,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="352" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
         <v>16</v>
       </c>
@@ -20296,7 +20320,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="353" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
         <v>16</v>
       </c>
@@ -20346,7 +20370,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="354" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
         <v>16</v>
       </c>
@@ -20396,7 +20420,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="355" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
         <v>16</v>
       </c>
@@ -20446,7 +20470,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="356" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
         <v>16</v>
       </c>
@@ -20496,7 +20520,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="357" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
         <v>16</v>
       </c>
@@ -20546,7 +20570,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="358" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
         <v>16</v>
       </c>
@@ -20578,7 +20602,7 @@
         <v>1.117</v>
       </c>
     </row>
-    <row r="359" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
         <v>16</v>
       </c>
@@ -20637,7 +20661,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="360" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
         <v>16</v>
       </c>
@@ -20670,7 +20694,7 @@
       </c>
       <c r="S360"/>
     </row>
-    <row r="361" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
         <v>16</v>
       </c>
@@ -20720,7 +20744,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="362" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
         <v>16</v>
       </c>
@@ -20762,7 +20786,7 @@
       </c>
       <c r="S362"/>
     </row>
-    <row r="363" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
         <v>16</v>
       </c>
@@ -20812,7 +20836,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="364" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
         <v>16</v>
       </c>
@@ -20854,7 +20878,7 @@
       </c>
       <c r="S364"/>
     </row>
-    <row r="365" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
         <v>16</v>
       </c>
@@ -20887,7 +20911,7 @@
       </c>
       <c r="S365"/>
     </row>
-    <row r="366" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
         <v>16</v>
       </c>
@@ -20920,7 +20944,7 @@
       </c>
       <c r="S366"/>
     </row>
-    <row r="367" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
         <v>16</v>
       </c>
@@ -20953,7 +20977,7 @@
       </c>
       <c r="S367"/>
     </row>
-    <row r="368" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
         <v>16</v>
       </c>
@@ -20985,7 +21009,7 @@
         <v>1.075</v>
       </c>
     </row>
-    <row r="369" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
         <v>16</v>
       </c>
@@ -21035,7 +21059,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="370" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
         <v>16</v>
       </c>
@@ -21085,7 +21109,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="371" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
         <v>16</v>
       </c>
@@ -21127,7 +21151,7 @@
       </c>
       <c r="S371"/>
     </row>
-    <row r="372" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
         <v>16</v>
       </c>
@@ -21177,7 +21201,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="373" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
         <v>16</v>
       </c>
@@ -21227,7 +21251,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="374" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
         <v>16</v>
       </c>
@@ -21277,7 +21301,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="375" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
         <v>16</v>
       </c>
@@ -21327,7 +21351,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="376" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
         <v>16</v>
       </c>
@@ -21377,7 +21401,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="377" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
         <v>16</v>
       </c>
@@ -21419,7 +21443,7 @@
       </c>
       <c r="S377"/>
     </row>
-    <row r="378" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
         <v>16</v>
       </c>
@@ -21469,7 +21493,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="379" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
         <v>16</v>
       </c>
@@ -21511,7 +21535,7 @@
       </c>
       <c r="S379"/>
     </row>
-    <row r="380" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
         <v>16</v>
       </c>
@@ -21553,7 +21577,7 @@
       </c>
       <c r="S380"/>
     </row>
-    <row r="381" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
         <v>16</v>
       </c>
@@ -21595,7 +21619,7 @@
       </c>
       <c r="S381"/>
     </row>
-    <row r="382" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
         <v>16</v>
       </c>
@@ -21636,7 +21660,7 @@
         <v>1.161</v>
       </c>
     </row>
-    <row r="383" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
         <v>16</v>
       </c>
@@ -21678,7 +21702,7 @@
       </c>
       <c r="S383"/>
     </row>
-    <row r="384" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
         <v>16</v>
       </c>
@@ -21720,7 +21744,7 @@
       </c>
       <c r="S384"/>
     </row>
-    <row r="385" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
         <v>16</v>
       </c>
@@ -21762,7 +21786,7 @@
       </c>
       <c r="S385"/>
     </row>
-    <row r="386" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
         <v>16</v>
       </c>
@@ -21812,7 +21836,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="387" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
         <v>16</v>
       </c>
@@ -21862,7 +21886,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="388" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
         <v>16</v>
       </c>
@@ -21912,7 +21936,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="389" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
         <v>16</v>
       </c>
@@ -21962,7 +21986,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="390" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
         <v>16</v>
       </c>
@@ -22004,7 +22028,7 @@
       </c>
       <c r="S390"/>
     </row>
-    <row r="391" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
         <v>16</v>
       </c>
@@ -22046,7 +22070,7 @@
       </c>
       <c r="S391"/>
     </row>
-    <row r="392" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
         <v>16</v>
       </c>
@@ -22096,7 +22120,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="393" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
         <v>16</v>
       </c>
@@ -22138,7 +22162,7 @@
       </c>
       <c r="S393"/>
     </row>
-    <row r="394" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
         <v>16</v>
       </c>
@@ -22171,7 +22195,7 @@
       </c>
       <c r="S394"/>
     </row>
-    <row r="395" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
         <v>16</v>
       </c>
@@ -22213,7 +22237,7 @@
       </c>
       <c r="S395"/>
     </row>
-    <row r="396" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
         <v>16</v>
       </c>
@@ -22263,7 +22287,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="397" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
         <v>16</v>
       </c>
@@ -22307,7 +22331,7 @@
         <v>894</v>
       </c>
     </row>
-    <row r="398" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
         <v>16</v>
       </c>
@@ -22357,7 +22381,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="399" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
         <v>16</v>
       </c>
@@ -22389,7 +22413,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="400" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
         <v>16</v>
       </c>
@@ -22421,7 +22445,7 @@
         <v>681</v>
       </c>
     </row>
-    <row r="401" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>16</v>
       </c>
@@ -22471,7 +22495,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="402" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>16</v>
       </c>
@@ -22521,7 +22545,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="403" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>16</v>
       </c>
@@ -22571,7 +22595,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="404" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>16</v>
       </c>
@@ -22612,7 +22636,7 @@
         <v>1.1060000000000001</v>
       </c>
     </row>
-    <row r="405" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>16</v>
       </c>
@@ -22662,7 +22686,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="406" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>16</v>
       </c>
@@ -22704,7 +22728,7 @@
       </c>
       <c r="S406"/>
     </row>
-    <row r="407" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>16</v>
       </c>
@@ -22746,7 +22770,7 @@
       </c>
       <c r="S407"/>
     </row>
-    <row r="408" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>16</v>
       </c>
@@ -22788,7 +22812,7 @@
       </c>
       <c r="S408"/>
     </row>
-    <row r="409" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>16</v>
       </c>
@@ -22838,7 +22862,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="410" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
         <v>16</v>
       </c>
@@ -22880,7 +22904,7 @@
       </c>
       <c r="S410"/>
     </row>
-    <row r="411" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
         <v>16</v>
       </c>
@@ -22930,7 +22954,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="412" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
         <v>16</v>
       </c>
@@ -22971,7 +22995,7 @@
         <v>756</v>
       </c>
     </row>
-    <row r="413" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
         <v>16</v>
       </c>
@@ -23013,7 +23037,7 @@
       </c>
       <c r="S413"/>
     </row>
-    <row r="414" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
         <v>16</v>
       </c>
@@ -23064,7 +23088,7 @@
       </c>
       <c r="S414"/>
     </row>
-    <row r="415" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
         <v>16</v>
       </c>
@@ -23106,7 +23130,7 @@
       </c>
       <c r="S415"/>
     </row>
-    <row r="416" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
         <v>16</v>
       </c>
@@ -23148,7 +23172,7 @@
       </c>
       <c r="S416"/>
     </row>
-    <row r="417" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
         <v>16</v>
       </c>
@@ -23198,7 +23222,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="418" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
         <v>16</v>
       </c>
@@ -23248,7 +23272,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="419" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
         <v>16</v>
       </c>
@@ -23289,7 +23313,7 @@
         <v>1.0649999999999999</v>
       </c>
     </row>
-    <row r="420" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
         <v>16</v>
       </c>
@@ -23331,7 +23355,7 @@
       </c>
       <c r="S420"/>
     </row>
-    <row r="421" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
         <v>16</v>
       </c>
@@ -23381,7 +23405,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="422" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
         <v>16</v>
       </c>
@@ -23431,7 +23455,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="423" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
         <v>16</v>
       </c>
@@ -23473,7 +23497,7 @@
       </c>
       <c r="S423"/>
     </row>
-    <row r="424" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
         <v>16</v>
       </c>
@@ -23523,7 +23547,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="425" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
         <v>16</v>
       </c>
@@ -23565,7 +23589,7 @@
       </c>
       <c r="S425"/>
     </row>
-    <row r="426" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
         <v>16</v>
       </c>
@@ -23615,7 +23639,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="427" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
         <v>16</v>
       </c>
@@ -23657,7 +23681,7 @@
       </c>
       <c r="S427"/>
     </row>
-    <row r="428" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
         <v>16</v>
       </c>
@@ -23699,7 +23723,7 @@
       </c>
       <c r="S428"/>
     </row>
-    <row r="429" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
         <v>16</v>
       </c>
@@ -23749,7 +23773,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="430" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
         <v>16</v>
       </c>
@@ -23791,7 +23815,7 @@
       </c>
       <c r="S430"/>
     </row>
-    <row r="431" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
         <v>16</v>
       </c>
@@ -23824,7 +23848,7 @@
       </c>
       <c r="S431"/>
     </row>
-    <row r="432" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
         <v>16</v>
       </c>
@@ -23866,7 +23890,7 @@
       </c>
       <c r="S432"/>
     </row>
-    <row r="433" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
         <v>16</v>
       </c>
@@ -23908,7 +23932,7 @@
       </c>
       <c r="S433"/>
     </row>
-    <row r="434" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
         <v>16</v>
       </c>
@@ -23958,7 +23982,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="435" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
         <v>16</v>
       </c>
@@ -24009,7 +24033,7 @@
       </c>
       <c r="S435"/>
     </row>
-    <row r="436" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
         <v>16</v>
       </c>
@@ -24059,7 +24083,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="437" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
         <v>16</v>
       </c>
@@ -24092,7 +24116,7 @@
       </c>
       <c r="S437"/>
     </row>
-    <row r="438" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
         <v>16</v>
       </c>
@@ -24134,7 +24158,7 @@
       </c>
       <c r="S438"/>
     </row>
-    <row r="439" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
         <v>16</v>
       </c>
@@ -24176,7 +24200,7 @@
       </c>
       <c r="S439"/>
     </row>
-    <row r="440" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
         <v>16</v>
       </c>
@@ -24218,7 +24242,7 @@
       </c>
       <c r="S440"/>
     </row>
-    <row r="441" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
         <v>16</v>
       </c>
@@ -24242,7 +24266,7 @@
       </c>
       <c r="S441"/>
     </row>
-    <row r="442" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
         <v>16</v>
       </c>
@@ -24284,7 +24308,7 @@
       </c>
       <c r="S442"/>
     </row>
-    <row r="443" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
         <v>16</v>
       </c>
@@ -24308,7 +24332,7 @@
       </c>
       <c r="S443"/>
     </row>
-    <row r="444" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
         <v>16</v>
       </c>
@@ -24349,7 +24373,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="445" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
         <v>16</v>
       </c>
@@ -24399,7 +24423,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="446" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
         <v>16</v>
       </c>
@@ -24449,7 +24473,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="447" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
         <v>16</v>
       </c>
@@ -24491,7 +24515,7 @@
       </c>
       <c r="S447"/>
     </row>
-    <row r="448" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
         <v>16</v>
       </c>
@@ -24541,7 +24565,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="449" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
         <v>16</v>
       </c>
@@ -24582,7 +24606,7 @@
         <v>1.147</v>
       </c>
     </row>
-    <row r="450" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
         <v>16</v>
       </c>
@@ -24623,7 +24647,7 @@
         <v>1.3280000000000001</v>
       </c>
     </row>
-    <row r="451" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
         <v>16</v>
       </c>
@@ -24665,7 +24689,7 @@
       </c>
       <c r="S451"/>
     </row>
-    <row r="452" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
         <v>16</v>
       </c>
@@ -24707,7 +24731,7 @@
       </c>
       <c r="S452"/>
     </row>
-    <row r="453" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
         <v>16</v>
       </c>
@@ -24740,7 +24764,7 @@
       </c>
       <c r="S453"/>
     </row>
-    <row r="454" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
         <v>16</v>
       </c>
@@ -24790,7 +24814,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="455" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
         <v>16</v>
       </c>
@@ -24831,7 +24855,7 @@
         <v>1.046</v>
       </c>
     </row>
-    <row r="456" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
         <v>16</v>
       </c>
@@ -24873,7 +24897,7 @@
       </c>
       <c r="S456"/>
     </row>
-    <row r="457" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
         <v>16</v>
       </c>
@@ -24923,7 +24947,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="458" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
         <v>16</v>
       </c>
@@ -24973,7 +24997,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="459" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
         <v>16</v>
       </c>
@@ -25023,7 +25047,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="460" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
         <v>16</v>
       </c>
@@ -25065,7 +25089,7 @@
       </c>
       <c r="S460"/>
     </row>
-    <row r="461" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
         <v>16</v>
       </c>
@@ -25107,7 +25131,7 @@
       </c>
       <c r="S461"/>
     </row>
-    <row r="462" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
         <v>16</v>
       </c>
@@ -25149,7 +25173,7 @@
       </c>
       <c r="S462"/>
     </row>
-    <row r="463" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
         <v>16</v>
       </c>
@@ -25199,7 +25223,7 @@
         <v>716</v>
       </c>
     </row>
-    <row r="464" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
         <v>16</v>
       </c>
@@ -25240,7 +25264,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="465" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
         <v>16</v>
       </c>
@@ -25281,7 +25305,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="466" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
         <v>16</v>
       </c>
@@ -25313,7 +25337,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="467" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
         <v>16</v>
       </c>
@@ -25355,7 +25379,7 @@
       </c>
       <c r="S467"/>
     </row>
-    <row r="468" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
         <v>16</v>
       </c>
@@ -25405,7 +25429,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="469" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
         <v>16</v>
       </c>
@@ -25446,7 +25470,7 @@
         <v>1.254</v>
       </c>
     </row>
-    <row r="470" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
         <v>16</v>
       </c>
@@ -25496,7 +25520,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="471" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
         <v>16</v>
       </c>
@@ -25546,7 +25570,7 @@
         <v>754</v>
       </c>
     </row>
-    <row r="472" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
         <v>16</v>
       </c>
@@ -25588,7 +25612,7 @@
       </c>
       <c r="S472"/>
     </row>
-    <row r="473" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
         <v>16</v>
       </c>
@@ -25629,7 +25653,7 @@
         <v>0.73399999999999999</v>
       </c>
     </row>
-    <row r="474" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
         <v>16</v>
       </c>
@@ -25662,7 +25686,7 @@
       </c>
       <c r="S474"/>
     </row>
-    <row r="475" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
         <v>16</v>
       </c>
@@ -25704,7 +25728,7 @@
       </c>
       <c r="S475"/>
     </row>
-    <row r="476" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
         <v>16</v>
       </c>
@@ -25746,7 +25770,7 @@
       </c>
       <c r="S476"/>
     </row>
-    <row r="477" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
         <v>16</v>
       </c>
@@ -25796,7 +25820,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="478" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
         <v>16</v>
       </c>
@@ -25837,7 +25861,7 @@
         <v>1.244</v>
       </c>
     </row>
-    <row r="479" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
         <v>16</v>
       </c>
@@ -25878,7 +25902,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="480" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
         <v>16</v>
       </c>
@@ -25920,7 +25944,7 @@
       </c>
       <c r="S480"/>
     </row>
-    <row r="481" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
         <v>16</v>
       </c>
@@ -25962,7 +25986,7 @@
       </c>
       <c r="S481"/>
     </row>
-    <row r="482" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:19" hidden="1" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
         <v>16</v>
       </c>
@@ -31958,7 +31982,9 @@
       <c r="R604">
         <v>2.5640000000000001</v>
       </c>
-      <c r="S604"/>
+      <c r="S604" t="s">
+        <v>896</v>
+      </c>
     </row>
     <row r="605" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A605" t="s">
@@ -35112,7 +35138,9 @@
       <c r="R679">
         <v>1.0449999999999999</v>
       </c>
-      <c r="S679"/>
+      <c r="S679" t="s">
+        <v>902</v>
+      </c>
     </row>
     <row r="680" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A680" t="s">
@@ -35604,7 +35632,9 @@
       <c r="R691">
         <v>1.0049999999999999</v>
       </c>
-      <c r="S691"/>
+      <c r="S691" t="s">
+        <v>901</v>
+      </c>
     </row>
     <row r="692" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A692" t="s">
@@ -36594,7 +36624,9 @@
       <c r="R714">
         <v>0.93200000000000005</v>
       </c>
-      <c r="S714"/>
+      <c r="S714" t="s">
+        <v>900</v>
+      </c>
     </row>
     <row r="715" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A715" t="s">
@@ -38200,7 +38232,7 @@
       </c>
       <c r="S752"/>
     </row>
-    <row r="753" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="753" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A753" t="s">
         <v>139</v>
       </c>
@@ -38240,8 +38272,9 @@
       <c r="R753">
         <v>0.95099999999999996</v>
       </c>
-    </row>
-    <row r="754" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S753"/>
+    </row>
+    <row r="754" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
         <v>139</v>
       </c>
@@ -38281,8 +38314,9 @@
       <c r="R754">
         <v>0.86499999999999999</v>
       </c>
-    </row>
-    <row r="755" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S754"/>
+    </row>
+    <row r="755" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A755" t="s">
         <v>139</v>
       </c>
@@ -38322,8 +38356,9 @@
       <c r="R755">
         <v>1.07</v>
       </c>
-    </row>
-    <row r="756" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S755"/>
+    </row>
+    <row r="756" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A756" t="s">
         <v>139</v>
       </c>
@@ -38363,8 +38398,9 @@
       <c r="R756">
         <v>1.169</v>
       </c>
-    </row>
-    <row r="757" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S756"/>
+    </row>
+    <row r="757" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A757" t="s">
         <v>139</v>
       </c>
@@ -38404,8 +38440,9 @@
       <c r="R757">
         <v>1.0489999999999999</v>
       </c>
-    </row>
-    <row r="758" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S757"/>
+    </row>
+    <row r="758" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A758" t="s">
         <v>139</v>
       </c>
@@ -38445,8 +38482,11 @@
       <c r="R758">
         <v>0.998</v>
       </c>
-    </row>
-    <row r="759" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S758" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="759" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A759" t="s">
         <v>139</v>
       </c>
@@ -38486,8 +38526,9 @@
       <c r="R759">
         <v>1.022</v>
       </c>
-    </row>
-    <row r="760" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S759"/>
+    </row>
+    <row r="760" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A760" t="s">
         <v>139</v>
       </c>
@@ -38527,8 +38568,9 @@
       <c r="R760">
         <v>1.419</v>
       </c>
-    </row>
-    <row r="761" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S760"/>
+    </row>
+    <row r="761" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A761" t="s">
         <v>139</v>
       </c>
@@ -38568,8 +38610,9 @@
       <c r="R761">
         <v>1.117</v>
       </c>
-    </row>
-    <row r="762" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S761"/>
+    </row>
+    <row r="762" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
         <v>139</v>
       </c>
@@ -38609,8 +38652,9 @@
       <c r="R762">
         <v>1.1000000000000001</v>
       </c>
-    </row>
-    <row r="763" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S762"/>
+    </row>
+    <row r="763" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A763" t="s">
         <v>139</v>
       </c>
@@ -38650,8 +38694,9 @@
       <c r="R763">
         <v>1.028</v>
       </c>
-    </row>
-    <row r="764" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S763"/>
+    </row>
+    <row r="764" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A764" t="s">
         <v>139</v>
       </c>
@@ -38691,8 +38736,9 @@
       <c r="R764">
         <v>1.613</v>
       </c>
-    </row>
-    <row r="765" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S764"/>
+    </row>
+    <row r="765" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
         <v>139</v>
       </c>
@@ -38732,8 +38778,9 @@
       <c r="R765">
         <v>0.93500000000000005</v>
       </c>
-    </row>
-    <row r="766" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S765"/>
+    </row>
+    <row r="766" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A766" t="s">
         <v>139</v>
       </c>
@@ -38773,8 +38820,9 @@
       <c r="R766">
         <v>1.042</v>
       </c>
-    </row>
-    <row r="767" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S766"/>
+    </row>
+    <row r="767" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A767" t="s">
         <v>139</v>
       </c>
@@ -38814,8 +38862,9 @@
       <c r="R767">
         <v>0.999</v>
       </c>
-    </row>
-    <row r="768" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="S767"/>
+    </row>
+    <row r="768" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A768" t="s">
         <v>139</v>
       </c>
@@ -38846,6 +38895,7 @@
       <c r="R768">
         <v>1.0640000000000001</v>
       </c>
+      <c r="S768"/>
     </row>
     <row r="769" spans="1:18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A769" t="s">
@@ -41812,7 +41862,9 @@
       <c r="R839">
         <v>0.63800000000000001</v>
       </c>
-      <c r="S839"/>
+      <c r="S839" t="s">
+        <v>898</v>
+      </c>
     </row>
     <row r="840" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A840" t="s">
@@ -49271,7 +49323,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1037" xr:uid="{29751ECF-5867-4DFC-949B-BE61CEB11EBC}"/>
+  <autoFilter ref="A1:S1037" xr:uid="{29751ECF-5867-4DFC-949B-BE61CEB11EBC}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="e"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>